<commit_message>
added ZW new rules
</commit_message>
<xml_diff>
--- a/output/CLFS_newformat_validation_report.xlsx
+++ b/output/CLFS_newformat_validation_report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,17 +462,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>RULE 19</t>
+          <t>HW_003</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>At any point in the last 12 months, were you self-employed? &amp; At any point in the last 12 months, did you work on your own (i.e., without paid employees) while running your own business or trade? &amp; Did you perform any freelance or assignment-based work via any of the following online platform(s) in the last 12 months?</t>
+          <t>Usual hours of work</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Freelance selected but self-employed/own-account not both Yes</t>
+          <t>SSOC major group 4-9: usual hours must be &gt;10 and &lt;25</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -482,17 +482,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RULE 6</t>
+          <t>RULE 19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>How much dividends and interests did you receive from other investment sources (e.g., bonds, shares, unit trust, personal loans to persons outside your households) in the last 12 months?</t>
+          <t>At any point in the last 12 months, were you self-employed? &amp; At any point in the last 12 months, did you work on your own (i.e., without paid employees) while running your own business or trade? &amp; Did you perform any freelance or assignment-based work via any of the following online platform(s) in the last 12 months?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Invalid dividends/other investment interest. Must be numeric between 0 and 50 (decimals allowed).</t>
+          <t>Freelance selected but self-employed/own-account not both Yes</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -502,20 +502,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>RULE 6</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>How much dividends and interests did you receive from other investment sources (e.g., bonds, shares, unit trust, personal loans to persons outside your households) in the last 12 months?</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Invalid dividends/other investment interest. Must be numeric between 0 and 50 (decimals allowed).</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>RULE 14</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>SSIC Code</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Unable to match SSIC Code from establishment name</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="D6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -530,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -787,17 +807,17 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>RULE 19</t>
+          <t>HW_003</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>At any point in the last 12 months, were you self-employed? &amp; At any point in the last 12 months, did you work on your own (i.e., without paid employees) while running your own business or trade? &amp; Did you perform any freelance or assignment-based work via any of the following online platform(s) in the last 12 months?</t>
+          <t>Usual hours of work</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Freelance selected but self-employed/own-account not both Yes</t>
+          <t>SSOC major group 4-9: usual hours must be &gt;10 and &lt;25</t>
         </is>
       </c>
     </row>
@@ -816,26 +836,26 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>6yyyy</t>
+          <t>ooo</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>RULE 5</t>
+          <t>RULE 19</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>How much interest did you receive from savings (e.g., current and saving accounts, fixed deposits) in the last 12 months?</t>
+          <t>At any point in the last 12 months, were you self-employed? &amp; At any point in the last 12 months, did you work on your own (i.e., without paid employees) while running your own business or trade? &amp; Did you perform any freelance or assignment-based work via any of the following online platform(s) in the last 12 months?</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Invalid interest. Must be numeric between 0 and 10 (decimals allowed).</t>
+          <t>Freelance selected but self-employed/own-account not both Yes</t>
         </is>
       </c>
     </row>
@@ -863,17 +883,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>RULE 6</t>
+          <t>RULE 5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>How much dividends and interests did you receive from other investment sources (e.g., bonds, shares, unit trust, personal loans to persons outside your households) in the last 12 months?</t>
+          <t>How much interest did you receive from savings (e.g., current and saving accounts, fixed deposits) in the last 12 months?</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Invalid dividends/other investment interest. Must be numeric between 0 and 50 (decimals allowed).</t>
+          <t>Invalid interest. Must be numeric between 0 and 10 (decimals allowed).</t>
         </is>
       </c>
     </row>
@@ -901,15 +921,91 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>RULE 6</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>How much dividends and interests did you receive from other investment sources (e.g., bonds, shares, unit trust, personal loans to persons outside your households) in the last 12 months?</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Invalid dividends/other investment interest. Must be numeric between 0 and 50 (decimals allowed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>CLFS_newformat.csv</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>69a55c77547674700bb3c52e</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>6yyyy</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>HW_003</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Usual hours of work</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>SSOC major group 4-9: usual hours must be &gt;10 and &lt;25</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CLFS_newformat.csv</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>69a55c77547674700bb3c52e</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>6yyyy</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>RULE 19</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>At any point in the last 12 months, were you self-employed? &amp; At any point in the last 12 months, did you work on your own (i.e., without paid employees) while running your own business or trade? &amp; Did you perform any freelance or assignment-based work via any of the following online platform(s) in the last 12 months?</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Freelance selected but self-employed/own-account not both Yes</t>
         </is>

</xml_diff>